<commit_message>
Escala: grupo C inicia em 01/11 (ordem C, D, A, B)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013CBcPNynpJREtonuZTCeAo
</commit_message>
<xml_diff>
--- a/Escala_48x144_Nov-Dez_2026.xlsx
+++ b/Escala_48x144_Nov-Dez_2026.xlsx
@@ -69,7 +69,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -91,11 +91,44 @@
         <color rgb="00808080"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -115,6 +148,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -480,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF27"/>
+  <dimension ref="A1:AG27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -687,8 +721,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="5" t="n"/>
+      <c r="A3" s="9" t="n"/>
+      <c r="B3" s="9" t="n"/>
       <c r="C3" s="3" t="n">
         <v>1</v>
       </c>
@@ -798,68 +832,68 @@
           <t>Comandante</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
       <c r="E5" s="7" t="n"/>
       <c r="F5" s="7" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="7" t="n"/>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="n"/>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="K5" s="7" t="n"/>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7" t="n"/>
       <c r="N5" s="7" t="n"/>
-      <c r="O5" s="7" t="n"/>
-      <c r="P5" s="7" t="n"/>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="P5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Q5" s="7" t="n"/>
       <c r="R5" s="7" t="n"/>
-      <c r="S5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="T5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="S5" s="7" t="n"/>
+      <c r="T5" s="7" t="n"/>
       <c r="U5" s="7" t="n"/>
       <c r="V5" s="7" t="n"/>
-      <c r="W5" s="7" t="n"/>
-      <c r="X5" s="7" t="n"/>
+      <c r="W5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="X5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Y5" s="7" t="n"/>
       <c r="Z5" s="7" t="n"/>
-      <c r="AA5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AB5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AA5" s="7" t="n"/>
+      <c r="AB5" s="7" t="n"/>
       <c r="AC5" s="7" t="n"/>
       <c r="AD5" s="7" t="n"/>
-      <c r="AE5" s="7" t="n"/>
-      <c r="AF5" s="7" t="n"/>
+      <c r="AE5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AF5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -872,68 +906,68 @@
           <t>Motorista</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="n"/>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="7" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="7" t="n"/>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
       <c r="M6" s="7" t="n"/>
       <c r="N6" s="7" t="n"/>
-      <c r="O6" s="7" t="n"/>
-      <c r="P6" s="7" t="n"/>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="P6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Q6" s="7" t="n"/>
       <c r="R6" s="7" t="n"/>
-      <c r="S6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="T6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="S6" s="7" t="n"/>
+      <c r="T6" s="7" t="n"/>
       <c r="U6" s="7" t="n"/>
       <c r="V6" s="7" t="n"/>
-      <c r="W6" s="7" t="n"/>
-      <c r="X6" s="7" t="n"/>
+      <c r="W6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="X6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Y6" s="7" t="n"/>
       <c r="Z6" s="7" t="n"/>
-      <c r="AA6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AB6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AA6" s="7" t="n"/>
+      <c r="AB6" s="7" t="n"/>
       <c r="AC6" s="7" t="n"/>
       <c r="AD6" s="7" t="n"/>
-      <c r="AE6" s="7" t="n"/>
-      <c r="AF6" s="7" t="n"/>
+      <c r="AE6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AF6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -946,68 +980,68 @@
           <t>Patrulheiro</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="L7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="n"/>
       <c r="N7" s="7" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="7" t="n"/>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Q7" s="7" t="n"/>
       <c r="R7" s="7" t="n"/>
-      <c r="S7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="T7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="S7" s="7" t="n"/>
+      <c r="T7" s="7" t="n"/>
       <c r="U7" s="7" t="n"/>
       <c r="V7" s="7" t="n"/>
-      <c r="W7" s="7" t="n"/>
-      <c r="X7" s="7" t="n"/>
+      <c r="W7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="X7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Y7" s="7" t="n"/>
       <c r="Z7" s="7" t="n"/>
-      <c r="AA7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AB7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AA7" s="7" t="n"/>
+      <c r="AB7" s="7" t="n"/>
       <c r="AC7" s="7" t="n"/>
       <c r="AD7" s="7" t="n"/>
-      <c r="AE7" s="7" t="n"/>
-      <c r="AF7" s="7" t="n"/>
+      <c r="AE7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AF7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1020,68 +1054,68 @@
           <t>Patrulheiro</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
       <c r="M8" s="7" t="n"/>
       <c r="N8" s="7" t="n"/>
-      <c r="O8" s="7" t="n"/>
-      <c r="P8" s="7" t="n"/>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="P8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Q8" s="7" t="n"/>
       <c r="R8" s="7" t="n"/>
-      <c r="S8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="T8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="S8" s="7" t="n"/>
+      <c r="T8" s="7" t="n"/>
       <c r="U8" s="7" t="n"/>
       <c r="V8" s="7" t="n"/>
-      <c r="W8" s="7" t="n"/>
-      <c r="X8" s="7" t="n"/>
+      <c r="W8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="X8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Y8" s="7" t="n"/>
       <c r="Z8" s="7" t="n"/>
-      <c r="AA8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AB8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AA8" s="7" t="n"/>
+      <c r="AB8" s="7" t="n"/>
       <c r="AC8" s="7" t="n"/>
       <c r="AD8" s="7" t="n"/>
-      <c r="AE8" s="7" t="n"/>
-      <c r="AF8" s="7" t="n"/>
+      <c r="AE8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AF8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -1103,64 +1137,56 @@
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
       <c r="G10" s="7" t="n"/>
       <c r="H10" s="7" t="n"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="n"/>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="K10" s="7" t="n"/>
       <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="N10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="7" t="n"/>
       <c r="O10" s="7" t="n"/>
       <c r="P10" s="7" t="n"/>
-      <c r="Q10" s="7" t="n"/>
-      <c r="R10" s="7" t="n"/>
+      <c r="Q10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="R10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="S10" s="7" t="n"/>
       <c r="T10" s="7" t="n"/>
-      <c r="U10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="V10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="U10" s="7" t="n"/>
+      <c r="V10" s="7" t="n"/>
       <c r="W10" s="7" t="n"/>
       <c r="X10" s="7" t="n"/>
-      <c r="Y10" s="7" t="n"/>
-      <c r="Z10" s="7" t="n"/>
+      <c r="Y10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="Z10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AA10" s="7" t="n"/>
       <c r="AB10" s="7" t="n"/>
-      <c r="AC10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AD10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AC10" s="7" t="n"/>
+      <c r="AD10" s="7" t="n"/>
       <c r="AE10" s="7" t="n"/>
       <c r="AF10" s="7" t="n"/>
     </row>
@@ -1177,64 +1203,56 @@
       </c>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
       <c r="G11" s="7" t="n"/>
       <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="K11" s="7" t="n"/>
       <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="N11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="M11" s="7" t="n"/>
+      <c r="N11" s="7" t="n"/>
       <c r="O11" s="7" t="n"/>
       <c r="P11" s="7" t="n"/>
-      <c r="Q11" s="7" t="n"/>
-      <c r="R11" s="7" t="n"/>
+      <c r="Q11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="R11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="S11" s="7" t="n"/>
       <c r="T11" s="7" t="n"/>
-      <c r="U11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="V11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="U11" s="7" t="n"/>
+      <c r="V11" s="7" t="n"/>
       <c r="W11" s="7" t="n"/>
       <c r="X11" s="7" t="n"/>
-      <c r="Y11" s="7" t="n"/>
-      <c r="Z11" s="7" t="n"/>
+      <c r="Y11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="Z11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AA11" s="7" t="n"/>
       <c r="AB11" s="7" t="n"/>
-      <c r="AC11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AD11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AC11" s="7" t="n"/>
+      <c r="AD11" s="7" t="n"/>
       <c r="AE11" s="7" t="n"/>
       <c r="AF11" s="7" t="n"/>
     </row>
@@ -1251,64 +1269,56 @@
       </c>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="E12" s="7" t="n"/>
+      <c r="F12" s="7" t="n"/>
       <c r="G12" s="7" t="n"/>
       <c r="H12" s="7" t="n"/>
-      <c r="I12" s="7" t="n"/>
-      <c r="J12" s="7" t="n"/>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="K12" s="7" t="n"/>
       <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="N12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="7" t="n"/>
       <c r="O12" s="7" t="n"/>
       <c r="P12" s="7" t="n"/>
-      <c r="Q12" s="7" t="n"/>
-      <c r="R12" s="7" t="n"/>
+      <c r="Q12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="R12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="S12" s="7" t="n"/>
       <c r="T12" s="7" t="n"/>
-      <c r="U12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="V12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="U12" s="7" t="n"/>
+      <c r="V12" s="7" t="n"/>
       <c r="W12" s="7" t="n"/>
       <c r="X12" s="7" t="n"/>
-      <c r="Y12" s="7" t="n"/>
-      <c r="Z12" s="7" t="n"/>
+      <c r="Y12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="Z12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AA12" s="7" t="n"/>
       <c r="AB12" s="7" t="n"/>
-      <c r="AC12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AD12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AC12" s="7" t="n"/>
+      <c r="AD12" s="7" t="n"/>
       <c r="AE12" s="7" t="n"/>
       <c r="AF12" s="7" t="n"/>
     </row>
@@ -1325,64 +1335,56 @@
       </c>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="E13" s="7" t="n"/>
+      <c r="F13" s="7" t="n"/>
       <c r="G13" s="7" t="n"/>
       <c r="H13" s="7" t="n"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="n"/>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="K13" s="7" t="n"/>
       <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="N13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="7" t="n"/>
       <c r="O13" s="7" t="n"/>
       <c r="P13" s="7" t="n"/>
-      <c r="Q13" s="7" t="n"/>
-      <c r="R13" s="7" t="n"/>
+      <c r="Q13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="R13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="S13" s="7" t="n"/>
       <c r="T13" s="7" t="n"/>
-      <c r="U13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="V13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="U13" s="7" t="n"/>
+      <c r="V13" s="7" t="n"/>
       <c r="W13" s="7" t="n"/>
       <c r="X13" s="7" t="n"/>
-      <c r="Y13" s="7" t="n"/>
-      <c r="Z13" s="7" t="n"/>
+      <c r="Y13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="Z13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AA13" s="7" t="n"/>
       <c r="AB13" s="7" t="n"/>
-      <c r="AC13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AD13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AC13" s="7" t="n"/>
+      <c r="AD13" s="7" t="n"/>
       <c r="AE13" s="7" t="n"/>
       <c r="AF13" s="7" t="n"/>
     </row>
@@ -1404,68 +1406,68 @@
           <t>Patrulheiro</t>
         </is>
       </c>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="E15" s="7" t="n"/>
       <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="7" t="n"/>
       <c r="I15" s="7" t="n"/>
       <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n"/>
-      <c r="L15" s="7" t="n"/>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="M15" s="7" t="n"/>
       <c r="N15" s="7" t="n"/>
-      <c r="O15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="P15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="O15" s="7" t="n"/>
+      <c r="P15" s="7" t="n"/>
       <c r="Q15" s="7" t="n"/>
       <c r="R15" s="7" t="n"/>
-      <c r="S15" s="7" t="n"/>
-      <c r="T15" s="7" t="n"/>
+      <c r="S15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="T15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="U15" s="7" t="n"/>
       <c r="V15" s="7" t="n"/>
-      <c r="W15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="X15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="W15" s="7" t="n"/>
+      <c r="X15" s="7" t="n"/>
       <c r="Y15" s="7" t="n"/>
       <c r="Z15" s="7" t="n"/>
-      <c r="AA15" s="7" t="n"/>
-      <c r="AB15" s="7" t="n"/>
+      <c r="AA15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AB15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AC15" s="7" t="n"/>
       <c r="AD15" s="7" t="n"/>
-      <c r="AE15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AF15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AE15" s="7" t="n"/>
+      <c r="AF15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1478,68 +1480,68 @@
           <t>Motorista</t>
         </is>
       </c>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="H16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
       <c r="I16" s="7" t="n"/>
       <c r="J16" s="7" t="n"/>
-      <c r="K16" s="7" t="n"/>
-      <c r="L16" s="7" t="n"/>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="M16" s="7" t="n"/>
       <c r="N16" s="7" t="n"/>
-      <c r="O16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="P16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="O16" s="7" t="n"/>
+      <c r="P16" s="7" t="n"/>
       <c r="Q16" s="7" t="n"/>
       <c r="R16" s="7" t="n"/>
-      <c r="S16" s="7" t="n"/>
-      <c r="T16" s="7" t="n"/>
+      <c r="S16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="T16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="U16" s="7" t="n"/>
       <c r="V16" s="7" t="n"/>
-      <c r="W16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="X16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="W16" s="7" t="n"/>
+      <c r="X16" s="7" t="n"/>
       <c r="Y16" s="7" t="n"/>
       <c r="Z16" s="7" t="n"/>
-      <c r="AA16" s="7" t="n"/>
-      <c r="AB16" s="7" t="n"/>
+      <c r="AA16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AB16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AC16" s="7" t="n"/>
       <c r="AD16" s="7" t="n"/>
-      <c r="AE16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AF16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AE16" s="7" t="n"/>
+      <c r="AF16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1552,68 +1554,68 @@
           <t>Patrulheiro</t>
         </is>
       </c>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="G17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="M17" s="7" t="n"/>
       <c r="N17" s="7" t="n"/>
-      <c r="O17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="P17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="O17" s="7" t="n"/>
+      <c r="P17" s="7" t="n"/>
       <c r="Q17" s="7" t="n"/>
       <c r="R17" s="7" t="n"/>
-      <c r="S17" s="7" t="n"/>
-      <c r="T17" s="7" t="n"/>
+      <c r="S17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="U17" s="7" t="n"/>
       <c r="V17" s="7" t="n"/>
-      <c r="W17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="X17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="W17" s="7" t="n"/>
+      <c r="X17" s="7" t="n"/>
       <c r="Y17" s="7" t="n"/>
       <c r="Z17" s="7" t="n"/>
-      <c r="AA17" s="7" t="n"/>
-      <c r="AB17" s="7" t="n"/>
+      <c r="AA17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AB17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AC17" s="7" t="n"/>
       <c r="AD17" s="7" t="n"/>
-      <c r="AE17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AF17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AE17" s="7" t="n"/>
+      <c r="AF17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1626,68 +1628,68 @@
           <t>Patrulheiro</t>
         </is>
       </c>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
+      <c r="K18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="M18" s="7" t="n"/>
       <c r="N18" s="7" t="n"/>
-      <c r="O18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="P18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="O18" s="7" t="n"/>
+      <c r="P18" s="7" t="n"/>
       <c r="Q18" s="7" t="n"/>
       <c r="R18" s="7" t="n"/>
-      <c r="S18" s="7" t="n"/>
-      <c r="T18" s="7" t="n"/>
+      <c r="S18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="T18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="U18" s="7" t="n"/>
       <c r="V18" s="7" t="n"/>
-      <c r="W18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="X18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="W18" s="7" t="n"/>
+      <c r="X18" s="7" t="n"/>
       <c r="Y18" s="7" t="n"/>
       <c r="Z18" s="7" t="n"/>
-      <c r="AA18" s="7" t="n"/>
-      <c r="AB18" s="7" t="n"/>
+      <c r="AA18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AB18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AC18" s="7" t="n"/>
       <c r="AD18" s="7" t="n"/>
-      <c r="AE18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AF18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AE18" s="7" t="n"/>
+      <c r="AF18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -1709,56 +1711,64 @@
       </c>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="G20" s="7" t="n"/>
       <c r="H20" s="7" t="n"/>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="I20" s="7" t="n"/>
+      <c r="J20" s="7" t="n"/>
       <c r="K20" s="7" t="n"/>
       <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
-      <c r="N20" s="7" t="n"/>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="O20" s="7" t="n"/>
       <c r="P20" s="7" t="n"/>
-      <c r="Q20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="R20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Q20" s="7" t="n"/>
+      <c r="R20" s="7" t="n"/>
       <c r="S20" s="7" t="n"/>
       <c r="T20" s="7" t="n"/>
-      <c r="U20" s="7" t="n"/>
-      <c r="V20" s="7" t="n"/>
+      <c r="U20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="V20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="W20" s="7" t="n"/>
       <c r="X20" s="7" t="n"/>
-      <c r="Y20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="Z20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Y20" s="7" t="n"/>
+      <c r="Z20" s="7" t="n"/>
       <c r="AA20" s="7" t="n"/>
       <c r="AB20" s="7" t="n"/>
-      <c r="AC20" s="7" t="n"/>
-      <c r="AD20" s="7" t="n"/>
+      <c r="AC20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AD20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AE20" s="7" t="n"/>
       <c r="AF20" s="7" t="n"/>
     </row>
@@ -1775,56 +1785,64 @@
       </c>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="G21" s="7" t="n"/>
       <c r="H21" s="7" t="n"/>
-      <c r="I21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="I21" s="7" t="n"/>
+      <c r="J21" s="7" t="n"/>
       <c r="K21" s="7" t="n"/>
       <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="O21" s="7" t="n"/>
       <c r="P21" s="7" t="n"/>
-      <c r="Q21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="R21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Q21" s="7" t="n"/>
+      <c r="R21" s="7" t="n"/>
       <c r="S21" s="7" t="n"/>
       <c r="T21" s="7" t="n"/>
-      <c r="U21" s="7" t="n"/>
-      <c r="V21" s="7" t="n"/>
+      <c r="U21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="V21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="W21" s="7" t="n"/>
       <c r="X21" s="7" t="n"/>
-      <c r="Y21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="Z21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Y21" s="7" t="n"/>
+      <c r="Z21" s="7" t="n"/>
       <c r="AA21" s="7" t="n"/>
       <c r="AB21" s="7" t="n"/>
-      <c r="AC21" s="7" t="n"/>
-      <c r="AD21" s="7" t="n"/>
+      <c r="AC21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AD21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AE21" s="7" t="n"/>
       <c r="AF21" s="7" t="n"/>
     </row>
@@ -1841,56 +1859,64 @@
       </c>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="G22" s="7" t="n"/>
       <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="I22" s="7" t="n"/>
+      <c r="J22" s="7" t="n"/>
       <c r="K22" s="7" t="n"/>
       <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="O22" s="7" t="n"/>
       <c r="P22" s="7" t="n"/>
-      <c r="Q22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="R22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Q22" s="7" t="n"/>
+      <c r="R22" s="7" t="n"/>
       <c r="S22" s="7" t="n"/>
       <c r="T22" s="7" t="n"/>
-      <c r="U22" s="7" t="n"/>
-      <c r="V22" s="7" t="n"/>
+      <c r="U22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="V22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="W22" s="7" t="n"/>
       <c r="X22" s="7" t="n"/>
-      <c r="Y22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="Z22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Y22" s="7" t="n"/>
+      <c r="Z22" s="7" t="n"/>
       <c r="AA22" s="7" t="n"/>
       <c r="AB22" s="7" t="n"/>
-      <c r="AC22" s="7" t="n"/>
-      <c r="AD22" s="7" t="n"/>
+      <c r="AC22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AD22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AE22" s="7" t="n"/>
       <c r="AF22" s="7" t="n"/>
     </row>
@@ -1985,10 +2011,11 @@
       <c r="AE25" s="7" t="n"/>
       <c r="AF25" s="7" t="n"/>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>F1 = dia de serviço (48h de serviço / 144h de folga). Ciclo: A 01–02/11, B 03–04, C 05–06, D 07–08, e repete.</t>
+          <t>F1 = dia de serviço (48h de serviço / 144h de folga). Ciclo: C 01–02/11, D 03–04, A 05–06, B 07–08, e repete.</t>
         </is>
       </c>
     </row>
@@ -2013,7 +2040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG27"/>
+  <dimension ref="A1:AH27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -2226,8 +2253,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n"/>
-      <c r="B3" s="5" t="n"/>
+      <c r="A3" s="9" t="n"/>
+      <c r="B3" s="9" t="n"/>
       <c r="C3" s="4" t="n">
         <v>1</v>
       </c>
@@ -2342,67 +2369,63 @@
       </c>
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="7" t="n"/>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
       <c r="G5" s="7" t="n"/>
       <c r="H5" s="7" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="K5" s="7" t="n"/>
       <c r="L5" s="7" t="n"/>
-      <c r="M5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="N5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="M5" s="7" t="n"/>
+      <c r="N5" s="7" t="n"/>
       <c r="O5" s="7" t="n"/>
       <c r="P5" s="7" t="n"/>
-      <c r="Q5" s="7" t="n"/>
-      <c r="R5" s="7" t="n"/>
+      <c r="Q5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="R5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="S5" s="7" t="n"/>
       <c r="T5" s="7" t="n"/>
-      <c r="U5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="V5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="U5" s="7" t="n"/>
+      <c r="V5" s="7" t="n"/>
       <c r="W5" s="7" t="n"/>
       <c r="X5" s="7" t="n"/>
-      <c r="Y5" s="7" t="n"/>
-      <c r="Z5" s="7" t="n"/>
+      <c r="Y5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="Z5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AA5" s="7" t="n"/>
       <c r="AB5" s="7" t="n"/>
-      <c r="AC5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AD5" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AC5" s="7" t="n"/>
+      <c r="AD5" s="7" t="n"/>
       <c r="AE5" s="7" t="n"/>
       <c r="AF5" s="7" t="n"/>
-      <c r="AG5" s="7" t="n"/>
+      <c r="AG5" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2417,67 +2440,63 @@
       </c>
       <c r="C6" s="7" t="n"/>
       <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
       <c r="G6" s="7" t="n"/>
       <c r="H6" s="7" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="K6" s="7" t="n"/>
       <c r="L6" s="7" t="n"/>
-      <c r="M6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="N6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="7" t="n"/>
       <c r="O6" s="7" t="n"/>
       <c r="P6" s="7" t="n"/>
-      <c r="Q6" s="7" t="n"/>
-      <c r="R6" s="7" t="n"/>
+      <c r="Q6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="R6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="S6" s="7" t="n"/>
       <c r="T6" s="7" t="n"/>
-      <c r="U6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="V6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="U6" s="7" t="n"/>
+      <c r="V6" s="7" t="n"/>
       <c r="W6" s="7" t="n"/>
       <c r="X6" s="7" t="n"/>
-      <c r="Y6" s="7" t="n"/>
-      <c r="Z6" s="7" t="n"/>
+      <c r="Y6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="Z6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AA6" s="7" t="n"/>
       <c r="AB6" s="7" t="n"/>
-      <c r="AC6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AD6" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AC6" s="7" t="n"/>
+      <c r="AD6" s="7" t="n"/>
       <c r="AE6" s="7" t="n"/>
       <c r="AF6" s="7" t="n"/>
-      <c r="AG6" s="7" t="n"/>
+      <c r="AG6" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2492,67 +2511,63 @@
       </c>
       <c r="C7" s="7" t="n"/>
       <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="n"/>
       <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="K7" s="7" t="n"/>
       <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="n"/>
       <c r="O7" s="7" t="n"/>
       <c r="P7" s="7" t="n"/>
-      <c r="Q7" s="7" t="n"/>
-      <c r="R7" s="7" t="n"/>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="R7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="S7" s="7" t="n"/>
       <c r="T7" s="7" t="n"/>
-      <c r="U7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="V7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="U7" s="7" t="n"/>
+      <c r="V7" s="7" t="n"/>
       <c r="W7" s="7" t="n"/>
       <c r="X7" s="7" t="n"/>
-      <c r="Y7" s="7" t="n"/>
-      <c r="Z7" s="7" t="n"/>
+      <c r="Y7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="Z7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AA7" s="7" t="n"/>
       <c r="AB7" s="7" t="n"/>
-      <c r="AC7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AD7" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AC7" s="7" t="n"/>
+      <c r="AD7" s="7" t="n"/>
       <c r="AE7" s="7" t="n"/>
       <c r="AF7" s="7" t="n"/>
-      <c r="AG7" s="7" t="n"/>
+      <c r="AG7" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2567,67 +2582,63 @@
       </c>
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
       <c r="G8" s="7" t="n"/>
       <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="N8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
       <c r="O8" s="7" t="n"/>
       <c r="P8" s="7" t="n"/>
-      <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="7" t="n"/>
+      <c r="Q8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="R8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="S8" s="7" t="n"/>
       <c r="T8" s="7" t="n"/>
-      <c r="U8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="V8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="7" t="n"/>
       <c r="W8" s="7" t="n"/>
       <c r="X8" s="7" t="n"/>
-      <c r="Y8" s="7" t="n"/>
-      <c r="Z8" s="7" t="n"/>
+      <c r="Y8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="Z8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AA8" s="7" t="n"/>
       <c r="AB8" s="7" t="n"/>
-      <c r="AC8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AD8" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AC8" s="7" t="n"/>
+      <c r="AD8" s="7" t="n"/>
       <c r="AE8" s="7" t="n"/>
       <c r="AF8" s="7" t="n"/>
-      <c r="AG8" s="7" t="n"/>
+      <c r="AG8" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -2647,68 +2658,68 @@
           <t>Comandante</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="n"/>
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
+      <c r="K10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="M10" s="7" t="n"/>
       <c r="N10" s="7" t="n"/>
-      <c r="O10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="P10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="O10" s="7" t="n"/>
+      <c r="P10" s="7" t="n"/>
       <c r="Q10" s="7" t="n"/>
       <c r="R10" s="7" t="n"/>
-      <c r="S10" s="7" t="n"/>
-      <c r="T10" s="7" t="n"/>
+      <c r="S10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="T10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="U10" s="7" t="n"/>
       <c r="V10" s="7" t="n"/>
-      <c r="W10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="X10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="W10" s="7" t="n"/>
+      <c r="X10" s="7" t="n"/>
       <c r="Y10" s="7" t="n"/>
       <c r="Z10" s="7" t="n"/>
-      <c r="AA10" s="7" t="n"/>
-      <c r="AB10" s="7" t="n"/>
+      <c r="AA10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AB10" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AC10" s="7" t="n"/>
       <c r="AD10" s="7" t="n"/>
-      <c r="AE10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AF10" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AE10" s="7" t="n"/>
+      <c r="AF10" s="7" t="n"/>
       <c r="AG10" s="7" t="n"/>
     </row>
     <row r="11">
@@ -2722,68 +2733,68 @@
           <t>Motorista</t>
         </is>
       </c>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
+      <c r="K11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="M11" s="7" t="n"/>
       <c r="N11" s="7" t="n"/>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="P11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="O11" s="7" t="n"/>
+      <c r="P11" s="7" t="n"/>
       <c r="Q11" s="7" t="n"/>
       <c r="R11" s="7" t="n"/>
-      <c r="S11" s="7" t="n"/>
-      <c r="T11" s="7" t="n"/>
+      <c r="S11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="U11" s="7" t="n"/>
       <c r="V11" s="7" t="n"/>
-      <c r="W11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="X11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="W11" s="7" t="n"/>
+      <c r="X11" s="7" t="n"/>
       <c r="Y11" s="7" t="n"/>
       <c r="Z11" s="7" t="n"/>
-      <c r="AA11" s="7" t="n"/>
-      <c r="AB11" s="7" t="n"/>
+      <c r="AA11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AB11" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AC11" s="7" t="n"/>
       <c r="AD11" s="7" t="n"/>
-      <c r="AE11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AF11" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AE11" s="7" t="n"/>
+      <c r="AF11" s="7" t="n"/>
       <c r="AG11" s="7" t="n"/>
     </row>
     <row r="12">
@@ -2797,68 +2808,68 @@
           <t>Motorista</t>
         </is>
       </c>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="G12" s="7" t="n"/>
+      <c r="H12" s="7" t="n"/>
       <c r="I12" s="7" t="n"/>
       <c r="J12" s="7" t="n"/>
-      <c r="K12" s="7" t="n"/>
-      <c r="L12" s="7" t="n"/>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="M12" s="7" t="n"/>
       <c r="N12" s="7" t="n"/>
-      <c r="O12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="P12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="7" t="n"/>
       <c r="Q12" s="7" t="n"/>
       <c r="R12" s="7" t="n"/>
-      <c r="S12" s="7" t="n"/>
-      <c r="T12" s="7" t="n"/>
+      <c r="S12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="T12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="U12" s="7" t="n"/>
       <c r="V12" s="7" t="n"/>
-      <c r="W12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="X12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="W12" s="7" t="n"/>
+      <c r="X12" s="7" t="n"/>
       <c r="Y12" s="7" t="n"/>
       <c r="Z12" s="7" t="n"/>
-      <c r="AA12" s="7" t="n"/>
-      <c r="AB12" s="7" t="n"/>
+      <c r="AA12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AB12" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AC12" s="7" t="n"/>
       <c r="AD12" s="7" t="n"/>
-      <c r="AE12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AF12" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AE12" s="7" t="n"/>
+      <c r="AF12" s="7" t="n"/>
       <c r="AG12" s="7" t="n"/>
     </row>
     <row r="13">
@@ -2872,68 +2883,68 @@
           <t>Patrulheiro</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="G13" s="7" t="n"/>
+      <c r="H13" s="7" t="n"/>
       <c r="I13" s="7" t="n"/>
       <c r="J13" s="7" t="n"/>
-      <c r="K13" s="7" t="n"/>
-      <c r="L13" s="7" t="n"/>
+      <c r="K13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="M13" s="7" t="n"/>
       <c r="N13" s="7" t="n"/>
-      <c r="O13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="P13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="7" t="n"/>
       <c r="Q13" s="7" t="n"/>
       <c r="R13" s="7" t="n"/>
-      <c r="S13" s="7" t="n"/>
-      <c r="T13" s="7" t="n"/>
+      <c r="S13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="U13" s="7" t="n"/>
       <c r="V13" s="7" t="n"/>
-      <c r="W13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="X13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="W13" s="7" t="n"/>
+      <c r="X13" s="7" t="n"/>
       <c r="Y13" s="7" t="n"/>
       <c r="Z13" s="7" t="n"/>
-      <c r="AA13" s="7" t="n"/>
-      <c r="AB13" s="7" t="n"/>
+      <c r="AA13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AB13" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AC13" s="7" t="n"/>
       <c r="AD13" s="7" t="n"/>
-      <c r="AE13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AF13" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AE13" s="7" t="n"/>
+      <c r="AF13" s="7" t="n"/>
       <c r="AG13" s="7" t="n"/>
     </row>
     <row r="14">
@@ -2956,63 +2967,67 @@
       </c>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="G15" s="7" t="n"/>
       <c r="H15" s="7" t="n"/>
-      <c r="I15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="I15" s="7" t="n"/>
+      <c r="J15" s="7" t="n"/>
       <c r="K15" s="7" t="n"/>
       <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7" t="n"/>
-      <c r="N15" s="7" t="n"/>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="O15" s="7" t="n"/>
       <c r="P15" s="7" t="n"/>
-      <c r="Q15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="R15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Q15" s="7" t="n"/>
+      <c r="R15" s="7" t="n"/>
       <c r="S15" s="7" t="n"/>
       <c r="T15" s="7" t="n"/>
-      <c r="U15" s="7" t="n"/>
-      <c r="V15" s="7" t="n"/>
+      <c r="U15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="V15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="W15" s="7" t="n"/>
       <c r="X15" s="7" t="n"/>
-      <c r="Y15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="Z15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Y15" s="7" t="n"/>
+      <c r="Z15" s="7" t="n"/>
       <c r="AA15" s="7" t="n"/>
       <c r="AB15" s="7" t="n"/>
-      <c r="AC15" s="7" t="n"/>
-      <c r="AD15" s="7" t="n"/>
+      <c r="AC15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AD15" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AE15" s="7" t="n"/>
       <c r="AF15" s="7" t="n"/>
-      <c r="AG15" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AG15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -3027,63 +3042,67 @@
       </c>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="7" t="n"/>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="G16" s="7" t="n"/>
       <c r="H16" s="7" t="n"/>
-      <c r="I16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="J16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="I16" s="7" t="n"/>
+      <c r="J16" s="7" t="n"/>
       <c r="K16" s="7" t="n"/>
       <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7" t="n"/>
-      <c r="N16" s="7" t="n"/>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="N16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="O16" s="7" t="n"/>
       <c r="P16" s="7" t="n"/>
-      <c r="Q16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="R16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Q16" s="7" t="n"/>
+      <c r="R16" s="7" t="n"/>
       <c r="S16" s="7" t="n"/>
       <c r="T16" s="7" t="n"/>
-      <c r="U16" s="7" t="n"/>
-      <c r="V16" s="7" t="n"/>
+      <c r="U16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="V16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="W16" s="7" t="n"/>
       <c r="X16" s="7" t="n"/>
-      <c r="Y16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="Z16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Y16" s="7" t="n"/>
+      <c r="Z16" s="7" t="n"/>
       <c r="AA16" s="7" t="n"/>
       <c r="AB16" s="7" t="n"/>
-      <c r="AC16" s="7" t="n"/>
-      <c r="AD16" s="7" t="n"/>
+      <c r="AC16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AD16" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AE16" s="7" t="n"/>
       <c r="AF16" s="7" t="n"/>
-      <c r="AG16" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AG16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -3098,63 +3117,67 @@
       </c>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="G17" s="7" t="n"/>
       <c r="H17" s="7" t="n"/>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="I17" s="7" t="n"/>
+      <c r="J17" s="7" t="n"/>
       <c r="K17" s="7" t="n"/>
       <c r="L17" s="7" t="n"/>
-      <c r="M17" s="7" t="n"/>
-      <c r="N17" s="7" t="n"/>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="O17" s="7" t="n"/>
       <c r="P17" s="7" t="n"/>
-      <c r="Q17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="R17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Q17" s="7" t="n"/>
+      <c r="R17" s="7" t="n"/>
       <c r="S17" s="7" t="n"/>
       <c r="T17" s="7" t="n"/>
-      <c r="U17" s="7" t="n"/>
-      <c r="V17" s="7" t="n"/>
+      <c r="U17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="V17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="W17" s="7" t="n"/>
       <c r="X17" s="7" t="n"/>
-      <c r="Y17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="Z17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Y17" s="7" t="n"/>
+      <c r="Z17" s="7" t="n"/>
       <c r="AA17" s="7" t="n"/>
       <c r="AB17" s="7" t="n"/>
-      <c r="AC17" s="7" t="n"/>
-      <c r="AD17" s="7" t="n"/>
+      <c r="AC17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AD17" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AE17" s="7" t="n"/>
       <c r="AF17" s="7" t="n"/>
-      <c r="AG17" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AG17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -3169,63 +3192,67 @@
       </c>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="G18" s="7" t="n"/>
       <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="n"/>
       <c r="K18" s="7" t="n"/>
       <c r="L18" s="7" t="n"/>
-      <c r="M18" s="7" t="n"/>
-      <c r="N18" s="7" t="n"/>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="O18" s="7" t="n"/>
       <c r="P18" s="7" t="n"/>
-      <c r="Q18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="R18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Q18" s="7" t="n"/>
+      <c r="R18" s="7" t="n"/>
       <c r="S18" s="7" t="n"/>
       <c r="T18" s="7" t="n"/>
-      <c r="U18" s="7" t="n"/>
-      <c r="V18" s="7" t="n"/>
+      <c r="U18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="V18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="W18" s="7" t="n"/>
       <c r="X18" s="7" t="n"/>
-      <c r="Y18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="Z18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="Y18" s="7" t="n"/>
+      <c r="Z18" s="7" t="n"/>
       <c r="AA18" s="7" t="n"/>
       <c r="AB18" s="7" t="n"/>
-      <c r="AC18" s="7" t="n"/>
-      <c r="AD18" s="7" t="n"/>
+      <c r="AC18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AD18" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AE18" s="7" t="n"/>
       <c r="AF18" s="7" t="n"/>
-      <c r="AG18" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AG18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -3245,68 +3272,68 @@
           <t>Comandante</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="L20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="K20" s="7" t="n"/>
+      <c r="L20" s="7" t="n"/>
       <c r="M20" s="7" t="n"/>
       <c r="N20" s="7" t="n"/>
-      <c r="O20" s="7" t="n"/>
-      <c r="P20" s="7" t="n"/>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="P20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Q20" s="7" t="n"/>
       <c r="R20" s="7" t="n"/>
-      <c r="S20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="T20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="S20" s="7" t="n"/>
+      <c r="T20" s="7" t="n"/>
       <c r="U20" s="7" t="n"/>
       <c r="V20" s="7" t="n"/>
-      <c r="W20" s="7" t="n"/>
-      <c r="X20" s="7" t="n"/>
+      <c r="W20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="X20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Y20" s="7" t="n"/>
       <c r="Z20" s="7" t="n"/>
-      <c r="AA20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AB20" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AA20" s="7" t="n"/>
+      <c r="AB20" s="7" t="n"/>
       <c r="AC20" s="7" t="n"/>
       <c r="AD20" s="7" t="n"/>
-      <c r="AE20" s="7" t="n"/>
-      <c r="AF20" s="7" t="n"/>
+      <c r="AE20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AF20" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AG20" s="7" t="n"/>
     </row>
     <row r="21">
@@ -3320,68 +3347,68 @@
           <t>Patrulheiro</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="I21" s="7" t="n"/>
       <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="L21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="K21" s="7" t="n"/>
+      <c r="L21" s="7" t="n"/>
       <c r="M21" s="7" t="n"/>
       <c r="N21" s="7" t="n"/>
-      <c r="O21" s="7" t="n"/>
-      <c r="P21" s="7" t="n"/>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Q21" s="7" t="n"/>
       <c r="R21" s="7" t="n"/>
-      <c r="S21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="T21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="S21" s="7" t="n"/>
+      <c r="T21" s="7" t="n"/>
       <c r="U21" s="7" t="n"/>
       <c r="V21" s="7" t="n"/>
-      <c r="W21" s="7" t="n"/>
-      <c r="X21" s="7" t="n"/>
+      <c r="W21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="X21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Y21" s="7" t="n"/>
       <c r="Z21" s="7" t="n"/>
-      <c r="AA21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AB21" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AA21" s="7" t="n"/>
+      <c r="AB21" s="7" t="n"/>
       <c r="AC21" s="7" t="n"/>
       <c r="AD21" s="7" t="n"/>
-      <c r="AE21" s="7" t="n"/>
-      <c r="AF21" s="7" t="n"/>
+      <c r="AE21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AF21" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AG21" s="7" t="n"/>
     </row>
     <row r="22">
@@ -3395,68 +3422,68 @@
           <t>Motorista</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="I22" s="7" t="n"/>
       <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="L22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="K22" s="7" t="n"/>
+      <c r="L22" s="7" t="n"/>
       <c r="M22" s="7" t="n"/>
       <c r="N22" s="7" t="n"/>
-      <c r="O22" s="7" t="n"/>
-      <c r="P22" s="7" t="n"/>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="P22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Q22" s="7" t="n"/>
       <c r="R22" s="7" t="n"/>
-      <c r="S22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="T22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="S22" s="7" t="n"/>
+      <c r="T22" s="7" t="n"/>
       <c r="U22" s="7" t="n"/>
       <c r="V22" s="7" t="n"/>
-      <c r="W22" s="7" t="n"/>
-      <c r="X22" s="7" t="n"/>
+      <c r="W22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="X22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="Y22" s="7" t="n"/>
       <c r="Z22" s="7" t="n"/>
-      <c r="AA22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="AB22" s="7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
+      <c r="AA22" s="7" t="n"/>
+      <c r="AB22" s="7" t="n"/>
       <c r="AC22" s="7" t="n"/>
       <c r="AD22" s="7" t="n"/>
-      <c r="AE22" s="7" t="n"/>
-      <c r="AF22" s="7" t="n"/>
+      <c r="AE22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="AF22" s="7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
       <c r="AG22" s="7" t="n"/>
     </row>
     <row r="23">
@@ -3552,10 +3579,11 @@
       <c r="AF25" s="7" t="n"/>
       <c r="AG25" s="7" t="n"/>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>F1 = dia de serviço (48h de serviço / 144h de folga). Ciclo: A 01–02/11, B 03–04, C 05–06, D 07–08, e repete.</t>
+          <t>F1 = dia de serviço (48h de serviço / 144h de folga). Ciclo: C 01–02/11, D 03–04, A 05–06, B 07–08, e repete.</t>
         </is>
       </c>
     </row>

</xml_diff>